<commit_message>
se agrego la liquidacion de horas
</commit_message>
<xml_diff>
--- a/date.xlsx
+++ b/date.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Lucas\Desktop\hikvision-hours-processor\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8F1BA4F7-B885-4A71-8880-71DB8557152B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B7F5E3A0-9FAD-4095-98EF-176D00922CB8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="172" uniqueCount="96">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="181" uniqueCount="97">
   <si>
     <t>Id</t>
   </si>
@@ -162,9 +162,6 @@
     <t>Zeller Lucas Ezequiel</t>
   </si>
   <si>
-    <t>lunes a miercoles</t>
-  </si>
-  <si>
     <t>Lencina Rocio Pilar</t>
   </si>
   <si>
@@ -322,6 +319,12 @@
   </si>
   <si>
     <t>ACCIDENTE DE TRABAJO</t>
+  </si>
+  <si>
+    <t>Todos</t>
+  </si>
+  <si>
+    <t>lunes , miercoles y viernes</t>
   </si>
 </sst>
 </file>
@@ -409,7 +412,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -442,6 +445,7 @@
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -587,7 +591,7 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="10"/>
                 <c:pt idx="0">
-                  <c:v>0</c:v>
+                  <c:v>1</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>0</c:v>
@@ -602,7 +606,7 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>0</c:v>
+                  <c:v>2</c:v>
                 </c:pt>
                 <c:pt idx="6">
                   <c:v>0</c:v>
@@ -757,7 +761,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="TablaEmpleados" displayName="TablaEmpleados" ref="A1:I29">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="TablaEmpleados" displayName="TablaEmpleados" ref="A1:I30">
   <tableColumns count="9">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Id"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Nombre"/>
@@ -951,14 +955,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:I1048570"/>
+  <dimension ref="A1:I1048571"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="10" style="1" customWidth="1"/>
     <col min="2" max="2" width="28" style="1" customWidth="1"/>
     <col min="3" max="6" width="18" style="1" customWidth="1"/>
     <col min="7" max="7" width="16" style="1" customWidth="1"/>
-    <col min="8" max="8" width="18" style="1" customWidth="1"/>
+    <col min="8" max="8" width="22.21875" style="1" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="20" style="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -991,53 +995,39 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:9" s="12" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A2" s="5">
-        <v>20</v>
+        <v>1</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="C2" s="3">
-        <v>0.3125</v>
-      </c>
-      <c r="D2" s="3">
-        <v>0.5</v>
-      </c>
-      <c r="E2" s="3">
-        <v>0.55208333333333337</v>
-      </c>
-      <c r="F2" s="3">
-        <v>0.73958333333333337</v>
-      </c>
-      <c r="G2" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="H2" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="I2" s="2" t="s">
-        <v>12</v>
-      </c>
+        <v>95</v>
+      </c>
+      <c r="C2" s="3"/>
+      <c r="D2" s="3"/>
+      <c r="E2" s="3"/>
+      <c r="F2" s="3"/>
+      <c r="G2" s="2"/>
+      <c r="H2" s="2"/>
+      <c r="I2" s="2"/>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A3" s="5">
-        <v>43</v>
+        <v>20</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="C3" s="3">
-        <v>0.27083333333333331</v>
+        <v>0.3125</v>
       </c>
       <c r="D3" s="3">
         <v>0.5</v>
       </c>
       <c r="E3" s="3">
-        <v>0.5625</v>
+        <v>0.55208333333333337</v>
       </c>
       <c r="F3" s="3">
-        <v>0.75</v>
+        <v>0.73958333333333337</v>
       </c>
       <c r="G3" s="2" t="s">
         <v>10</v>
@@ -1046,15 +1036,15 @@
         <v>11</v>
       </c>
       <c r="I3" s="2" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A4" s="5">
-        <v>51</v>
+        <v>43</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="C4" s="3">
         <v>0.27083333333333331</v>
@@ -1080,10 +1070,10 @@
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A5" s="5">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C5" s="3">
         <v>0.27083333333333331</v>
@@ -1109,10 +1099,10 @@
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A6" s="5">
-        <v>67</v>
+        <v>52</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C6" s="3">
         <v>0.27083333333333331</v>
@@ -1138,13 +1128,13 @@
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A7" s="5">
-        <v>79</v>
+        <v>67</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C7" s="3">
-        <v>0.3125</v>
+        <v>0.27083333333333331</v>
       </c>
       <c r="D7" s="3">
         <v>0.5</v>
@@ -1162,18 +1152,18 @@
         <v>11</v>
       </c>
       <c r="I7" s="2" t="s">
-        <v>19</v>
+        <v>14</v>
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A8" s="5">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="C8" s="3">
-        <v>0.27083333333333331</v>
+        <v>0.3125</v>
       </c>
       <c r="D8" s="3">
         <v>0.5</v>
@@ -1191,48 +1181,52 @@
         <v>11</v>
       </c>
       <c r="I8" s="2" t="s">
-        <v>14</v>
+        <v>19</v>
       </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A9" s="5">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C9" s="3">
-        <v>0.29166666666666669</v>
-      </c>
-      <c r="D9" s="3"/>
-      <c r="E9" s="3"/>
+        <v>0.27083333333333331</v>
+      </c>
+      <c r="D9" s="3">
+        <v>0.5</v>
+      </c>
+      <c r="E9" s="3">
+        <v>0.5625</v>
+      </c>
       <c r="F9" s="3">
-        <v>0.58333333333333337</v>
+        <v>0.75</v>
       </c>
       <c r="G9" s="2" t="s">
-        <v>22</v>
+        <v>10</v>
       </c>
       <c r="H9" s="2" t="s">
         <v>11</v>
       </c>
       <c r="I9" s="2" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A10" s="5">
-        <v>93</v>
+        <v>83</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="C10" s="3">
-        <v>0.33333333333333331</v>
+        <v>0.29166666666666669</v>
       </c>
       <c r="D10" s="3"/>
       <c r="E10" s="3"/>
       <c r="F10" s="3">
-        <v>0.54166666666666663</v>
+        <v>0.58333333333333337</v>
       </c>
       <c r="G10" s="2" t="s">
         <v>22</v>
@@ -1246,25 +1240,21 @@
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A11" s="5">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C11" s="3">
-        <v>0.3125</v>
-      </c>
-      <c r="D11" s="3">
-        <v>0.5</v>
-      </c>
-      <c r="E11" s="3">
-        <v>0.5625</v>
-      </c>
+        <v>0.33333333333333331</v>
+      </c>
+      <c r="D11" s="3"/>
+      <c r="E11" s="3"/>
       <c r="F11" s="3">
-        <v>0.75</v>
+        <v>0.54166666666666663</v>
       </c>
       <c r="G11" s="2" t="s">
-        <v>10</v>
+        <v>22</v>
       </c>
       <c r="H11" s="2" t="s">
         <v>11</v>
@@ -1275,10 +1265,10 @@
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A12" s="5">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C12" s="3">
         <v>0.3125</v>
@@ -1299,15 +1289,15 @@
         <v>11</v>
       </c>
       <c r="I12" s="2" t="s">
-        <v>19</v>
+        <v>12</v>
       </c>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A13" s="5">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C13" s="3">
         <v>0.3125</v>
@@ -1333,67 +1323,67 @@
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A14" s="5">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C14" s="3">
-        <v>0.33333333333333331</v>
-      </c>
-      <c r="D14" s="3"/>
-      <c r="E14" s="3"/>
+        <v>0.3125</v>
+      </c>
+      <c r="D14" s="3">
+        <v>0.5</v>
+      </c>
+      <c r="E14" s="3">
+        <v>0.5625</v>
+      </c>
       <c r="F14" s="3">
-        <v>0.58333333333333337</v>
+        <v>0.75</v>
       </c>
       <c r="G14" s="2" t="s">
-        <v>22</v>
+        <v>10</v>
       </c>
       <c r="H14" s="2" t="s">
         <v>11</v>
       </c>
       <c r="I14" s="2" t="s">
-        <v>12</v>
+        <v>19</v>
       </c>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A15" s="5">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C15" s="3">
-        <v>0.3125</v>
-      </c>
-      <c r="D15" s="3">
-        <v>0.5</v>
-      </c>
-      <c r="E15" s="3">
-        <v>0.5625</v>
-      </c>
+        <v>0.33333333333333331</v>
+      </c>
+      <c r="D15" s="3"/>
+      <c r="E15" s="3"/>
       <c r="F15" s="3">
-        <v>0.75</v>
+        <v>0.58333333333333337</v>
       </c>
       <c r="G15" s="2" t="s">
-        <v>10</v>
+        <v>22</v>
       </c>
       <c r="H15" s="2" t="s">
         <v>11</v>
       </c>
       <c r="I15" s="2" t="s">
-        <v>19</v>
+        <v>12</v>
       </c>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A16" s="5">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C16" s="3">
-        <v>0.27083333333333331</v>
+        <v>0.3125</v>
       </c>
       <c r="D16" s="3">
         <v>0.5</v>
@@ -1411,18 +1401,18 @@
         <v>11</v>
       </c>
       <c r="I16" s="2" t="s">
-        <v>14</v>
+        <v>19</v>
       </c>
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A17" s="5">
-        <v>105</v>
+        <v>101</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C17" s="3">
-        <v>0.3125</v>
+        <v>0.27083333333333331</v>
       </c>
       <c r="D17" s="3">
         <v>0.5</v>
@@ -1440,24 +1430,28 @@
         <v>11</v>
       </c>
       <c r="I17" s="2" t="s">
-        <v>19</v>
+        <v>14</v>
       </c>
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A18" s="5">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C18" s="3">
-        <v>0.33333333333333331</v>
+        <v>0.3125</v>
       </c>
       <c r="D18" s="3">
         <v>0.5</v>
       </c>
-      <c r="E18" s="3"/>
-      <c r="F18" s="3"/>
+      <c r="E18" s="3">
+        <v>0.5625</v>
+      </c>
+      <c r="F18" s="3">
+        <v>0.75</v>
+      </c>
       <c r="G18" s="2" t="s">
         <v>10</v>
       </c>
@@ -1465,69 +1459,65 @@
         <v>11</v>
       </c>
       <c r="I18" s="2" t="s">
-        <v>12</v>
+        <v>19</v>
       </c>
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A19" s="5">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C19" s="3">
-        <v>0.375</v>
-      </c>
-      <c r="D19" s="3"/>
+        <v>0.33333333333333331</v>
+      </c>
+      <c r="D19" s="3">
+        <v>0.5</v>
+      </c>
       <c r="E19" s="3"/>
-      <c r="F19" s="3">
-        <v>0.625</v>
-      </c>
+      <c r="F19" s="3"/>
       <c r="G19" s="2" t="s">
-        <v>22</v>
+        <v>10</v>
       </c>
       <c r="H19" s="2" t="s">
         <v>11</v>
       </c>
       <c r="I19" s="2" t="s">
-        <v>33</v>
+        <v>12</v>
       </c>
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A20" s="5">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="C20" s="3">
-        <v>0.27083333333333331</v>
-      </c>
-      <c r="D20" s="3">
-        <v>0.5</v>
-      </c>
-      <c r="E20" s="3">
-        <v>0.5625</v>
-      </c>
+        <v>0.375</v>
+      </c>
+      <c r="D20" s="3"/>
+      <c r="E20" s="3"/>
       <c r="F20" s="3">
-        <v>0.75</v>
+        <v>0.625</v>
       </c>
       <c r="G20" s="2" t="s">
-        <v>10</v>
+        <v>22</v>
       </c>
       <c r="H20" s="2" t="s">
         <v>11</v>
       </c>
       <c r="I20" s="2" t="s">
-        <v>14</v>
+        <v>33</v>
       </c>
     </row>
     <row r="21" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A21" s="5">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C21" s="3">
         <v>0.27083333333333331</v>
@@ -1553,13 +1543,13 @@
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A22" s="5">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C22" s="3">
-        <v>0.3125</v>
+        <v>0.27083333333333331</v>
       </c>
       <c r="D22" s="3">
         <v>0.5</v>
@@ -1577,15 +1567,15 @@
         <v>11</v>
       </c>
       <c r="I22" s="2" t="s">
-        <v>19</v>
+        <v>14</v>
       </c>
     </row>
     <row r="23" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A23" s="5">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C23" s="3">
         <v>0.3125</v>
@@ -1606,106 +1596,110 @@
         <v>11</v>
       </c>
       <c r="I23" s="2" t="s">
-        <v>33</v>
+        <v>19</v>
       </c>
     </row>
     <row r="24" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A24" s="5">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C24" s="3">
-        <v>0.33333333333333331</v>
+        <v>0.3125</v>
       </c>
       <c r="D24" s="3">
         <v>0.5</v>
       </c>
-      <c r="E24" s="3"/>
-      <c r="F24" s="3"/>
+      <c r="E24" s="3">
+        <v>0.5625</v>
+      </c>
+      <c r="F24" s="3">
+        <v>0.75</v>
+      </c>
       <c r="G24" s="2" t="s">
-        <v>22</v>
+        <v>10</v>
       </c>
       <c r="H24" s="2" t="s">
         <v>11</v>
       </c>
       <c r="I24" s="2" t="s">
-        <v>39</v>
+        <v>33</v>
       </c>
     </row>
     <row r="25" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A25" s="5">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="C25" s="3">
-        <v>0.27083333333333331</v>
+        <v>0.33333333333333331</v>
       </c>
       <c r="D25" s="3">
         <v>0.5</v>
       </c>
-      <c r="E25" s="3">
-        <v>0.5625</v>
-      </c>
-      <c r="F25" s="3">
-        <v>0.75</v>
-      </c>
-      <c r="G25" s="2"/>
+      <c r="E25" s="3"/>
+      <c r="F25" s="3"/>
+      <c r="G25" s="2" t="s">
+        <v>22</v>
+      </c>
       <c r="H25" s="2" t="s">
         <v>11</v>
       </c>
       <c r="I25" s="2" t="s">
-        <v>14</v>
+        <v>39</v>
       </c>
     </row>
     <row r="26" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A26" s="5">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C26" s="3">
-        <v>0.3125</v>
+        <v>0.27083333333333331</v>
       </c>
       <c r="D26" s="3">
         <v>0.5</v>
       </c>
-      <c r="E26" s="3"/>
-      <c r="F26" s="3"/>
-      <c r="G26" s="2" t="s">
-        <v>22</v>
-      </c>
+      <c r="E26" s="3">
+        <v>0.5625</v>
+      </c>
+      <c r="F26" s="3">
+        <v>0.75</v>
+      </c>
+      <c r="G26" s="2"/>
       <c r="H26" s="2" t="s">
-        <v>42</v>
+        <v>11</v>
       </c>
       <c r="I26" s="2" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
     </row>
     <row r="27" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A27" s="5">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C27" s="3">
-        <v>0.375</v>
-      </c>
-      <c r="D27" s="3"/>
+        <v>0.3125</v>
+      </c>
+      <c r="D27" s="3">
+        <v>0.5</v>
+      </c>
       <c r="E27" s="3"/>
-      <c r="F27" s="3">
-        <v>0.70833333333333337</v>
-      </c>
+      <c r="F27" s="3"/>
       <c r="G27" s="2" t="s">
         <v>22</v>
       </c>
       <c r="H27" s="2" t="s">
-        <v>11</v>
+        <v>96</v>
       </c>
       <c r="I27" s="2" t="s">
         <v>12</v>
@@ -1713,37 +1707,35 @@
     </row>
     <row r="28" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A28" s="5">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="C28" s="3">
-        <v>0.33333333333333331</v>
-      </c>
-      <c r="D28" s="3">
-        <v>0.5</v>
-      </c>
-      <c r="E28" s="3">
-        <v>0.58333333333333337</v>
-      </c>
+        <v>0.375</v>
+      </c>
+      <c r="D28" s="3"/>
+      <c r="E28" s="3"/>
       <c r="F28" s="3">
-        <v>0.75</v>
-      </c>
-      <c r="G28" s="2"/>
+        <v>0.70833333333333337</v>
+      </c>
+      <c r="G28" s="2" t="s">
+        <v>22</v>
+      </c>
       <c r="H28" s="2" t="s">
         <v>11</v>
       </c>
       <c r="I28" s="2" t="s">
-        <v>39</v>
+        <v>12</v>
       </c>
     </row>
     <row r="29" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A29" s="5">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="C29" s="3">
         <v>0.33333333333333331</v>
@@ -1765,8 +1757,35 @@
         <v>39</v>
       </c>
     </row>
-    <row r="1048570" spans="7:7" x14ac:dyDescent="0.3">
-      <c r="G1048570" s="2"/>
+    <row r="30" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A30" s="5">
+        <v>121</v>
+      </c>
+      <c r="B30" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="C30" s="3">
+        <v>0.33333333333333331</v>
+      </c>
+      <c r="D30" s="3">
+        <v>0.5</v>
+      </c>
+      <c r="E30" s="3">
+        <v>0.58333333333333337</v>
+      </c>
+      <c r="F30" s="3">
+        <v>0.75</v>
+      </c>
+      <c r="G30" s="2"/>
+      <c r="H30" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="I30" s="2" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="1048571" spans="7:7" x14ac:dyDescent="0.3">
+      <c r="G1048571" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1788,88 +1807,88 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A1" s="6" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B1" s="6"/>
       <c r="C1" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="E1" s="6" t="s">
         <v>47</v>
-      </c>
-      <c r="E1" s="6" t="s">
-        <v>48</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="C2" t="s">
+        <v>49</v>
+      </c>
+      <c r="E2" s="7" t="s">
         <v>50</v>
-      </c>
-      <c r="E2" s="7" t="s">
-        <v>51</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="C3" t="s">
+        <v>52</v>
+      </c>
+      <c r="E3" s="7" t="s">
         <v>53</v>
-      </c>
-      <c r="E3" s="7" t="s">
-        <v>54</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C4" t="s">
+        <v>55</v>
+      </c>
+      <c r="E4" s="7" t="s">
         <v>56</v>
-      </c>
-      <c r="E4" s="7" t="s">
-        <v>57</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="E5" s="7" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="E6" s="7" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
     </row>
   </sheetData>
@@ -1894,37 +1913,37 @@
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A1" s="11" t="s">
+        <v>66</v>
+      </c>
+      <c r="B1" s="11" t="s">
         <v>67</v>
       </c>
-      <c r="B1" s="11" t="s">
+      <c r="C1" s="11" t="s">
         <v>68</v>
       </c>
-      <c r="C1" s="11" t="s">
+      <c r="D1" s="11" t="s">
         <v>69</v>
       </c>
-      <c r="D1" s="11" t="s">
+      <c r="E1" s="11" t="s">
         <v>70</v>
       </c>
-      <c r="E1" s="11" t="s">
+      <c r="F1" s="11" t="s">
         <v>71</v>
       </c>
-      <c r="F1" s="11" t="s">
+      <c r="G1" s="11" t="s">
         <v>72</v>
       </c>
-      <c r="G1" s="11" t="s">
+      <c r="H1" s="11" t="s">
         <v>73</v>
       </c>
-      <c r="H1" s="11" t="s">
+      <c r="I1" s="11" t="s">
         <v>74</v>
       </c>
-      <c r="I1" s="11" t="s">
+      <c r="J1" s="11" t="s">
         <v>75</v>
       </c>
-      <c r="J1" s="11" t="s">
+      <c r="K1" s="11" t="s">
         <v>76</v>
-      </c>
-      <c r="K1" s="11" t="s">
-        <v>77</v>
       </c>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.3">
@@ -1944,7 +1963,7 @@
         <v>lunes a viernes</v>
       </c>
       <c r="E2" s="7" t="s">
-        <v>94</v>
+        <v>48</v>
       </c>
       <c r="F2" s="9">
         <v>46140</v>
@@ -1957,7 +1976,7 @@
         <v>1</v>
       </c>
       <c r="I2" s="7" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="J2" s="7"/>
       <c r="K2" s="7" t="str">
@@ -1966,127 +1985,155 @@
       </c>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A3" s="7"/>
+      <c r="A3" s="7">
+        <v>1</v>
+      </c>
       <c r="B3" s="7" t="str">
         <f>IF(A3="","",IFERROR(VLOOKUP(A3,Empleados!A:B,2,FALSE),""))</f>
-        <v/>
-      </c>
-      <c r="C3" s="7" t="str">
+        <v>Todos</v>
+      </c>
+      <c r="C3" s="7">
         <f>IF(A3="","",IFERROR(VLOOKUP(A3,Empleados!A:I,9,FALSE),""))</f>
-        <v/>
-      </c>
-      <c r="D3" s="7" t="str">
+        <v>0</v>
+      </c>
+      <c r="D3" s="7">
         <f>IF(A3="","",IFERROR(VLOOKUP(A3,Empleados!A:H,8,FALSE),""))</f>
-        <v/>
-      </c>
-      <c r="E3" s="7"/>
-      <c r="F3" s="9"/>
-      <c r="G3" s="9"/>
-      <c r="H3" s="10" t="str">
+        <v>0</v>
+      </c>
+      <c r="E3" s="7" t="s">
+        <v>61</v>
+      </c>
+      <c r="F3" s="9">
+        <v>46143</v>
+      </c>
+      <c r="G3" s="9">
+        <v>46143</v>
+      </c>
+      <c r="H3" s="10">
         <f t="shared" ref="H3:H66" si="1">IF(OR(F3="",G3=""),"",G3-F3+1)</f>
-        <v/>
-      </c>
-      <c r="I3" s="7" t="str">
-        <f t="shared" ref="I3:I66" si="2">IF(A3="","","PENDIENTE")</f>
-        <v/>
+        <v>1</v>
+      </c>
+      <c r="I3" s="7" t="s">
+        <v>52</v>
       </c>
       <c r="J3" s="7"/>
       <c r="K3" s="7" t="str">
         <f t="shared" si="0"/>
-        <v/>
+        <v>1|20260501|20260501</v>
       </c>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A4" s="7"/>
+      <c r="A4" s="7">
+        <v>1</v>
+      </c>
       <c r="B4" s="7" t="str">
         <f>IF(A4="","",IFERROR(VLOOKUP(A4,Empleados!A:B,2,FALSE),""))</f>
-        <v/>
-      </c>
-      <c r="C4" s="7" t="str">
+        <v>Todos</v>
+      </c>
+      <c r="C4" s="7">
         <f>IF(A4="","",IFERROR(VLOOKUP(A4,Empleados!A:I,9,FALSE),""))</f>
-        <v/>
-      </c>
-      <c r="D4" s="7" t="str">
+        <v>0</v>
+      </c>
+      <c r="D4" s="7">
         <f>IF(A4="","",IFERROR(VLOOKUP(A4,Empleados!A:H,8,FALSE),""))</f>
-        <v/>
-      </c>
-      <c r="E4" s="7"/>
-      <c r="F4" s="9"/>
-      <c r="G4" s="9"/>
-      <c r="H4" s="10" t="str">
+        <v>0</v>
+      </c>
+      <c r="E4" s="7" t="s">
+        <v>61</v>
+      </c>
+      <c r="F4" s="9">
+        <v>46167</v>
+      </c>
+      <c r="G4" s="9">
+        <v>46167</v>
+      </c>
+      <c r="H4" s="10">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="I4" s="7" t="str">
-        <f t="shared" si="2"/>
-        <v/>
+        <v>1</v>
+      </c>
+      <c r="I4" s="7" t="s">
+        <v>52</v>
       </c>
       <c r="J4" s="7"/>
       <c r="K4" s="7" t="str">
         <f t="shared" si="0"/>
-        <v/>
+        <v>1|20260525|20260525</v>
       </c>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A5" s="7"/>
+      <c r="A5" s="7">
+        <v>82</v>
+      </c>
       <c r="B5" s="7" t="str">
         <f>IF(A5="","",IFERROR(VLOOKUP(A5,Empleados!A:B,2,FALSE),""))</f>
-        <v/>
+        <v>Godoy Denis</v>
       </c>
       <c r="C5" s="7" t="str">
         <f>IF(A5="","",IFERROR(VLOOKUP(A5,Empleados!A:I,9,FALSE),""))</f>
-        <v/>
+        <v>Metalurgica</v>
       </c>
       <c r="D5" s="7" t="str">
         <f>IF(A5="","",IFERROR(VLOOKUP(A5,Empleados!A:H,8,FALSE),""))</f>
-        <v/>
-      </c>
-      <c r="E5" s="7"/>
-      <c r="F5" s="9"/>
-      <c r="G5" s="9"/>
-      <c r="H5" s="10" t="str">
+        <v>lunes a viernes</v>
+      </c>
+      <c r="E5" s="7" t="s">
+        <v>94</v>
+      </c>
+      <c r="F5" s="9">
+        <v>46146</v>
+      </c>
+      <c r="G5" s="9">
+        <v>46149</v>
+      </c>
+      <c r="H5" s="10">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="I5" s="7" t="str">
-        <f t="shared" si="2"/>
-        <v/>
+        <v>4</v>
+      </c>
+      <c r="I5" s="7" t="s">
+        <v>52</v>
       </c>
       <c r="J5" s="7"/>
       <c r="K5" s="7" t="str">
         <f t="shared" si="0"/>
-        <v/>
+        <v>82|20260504|20260507</v>
       </c>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A6" s="7"/>
+      <c r="A6" s="7">
+        <v>52</v>
+      </c>
       <c r="B6" s="7" t="str">
         <f>IF(A6="","",IFERROR(VLOOKUP(A6,Empleados!A:B,2,FALSE),""))</f>
-        <v/>
+        <v>Mario Butto</v>
       </c>
       <c r="C6" s="7" t="str">
         <f>IF(A6="","",IFERROR(VLOOKUP(A6,Empleados!A:I,9,FALSE),""))</f>
-        <v/>
+        <v>Metalurgica</v>
       </c>
       <c r="D6" s="7" t="str">
         <f>IF(A6="","",IFERROR(VLOOKUP(A6,Empleados!A:H,8,FALSE),""))</f>
-        <v/>
-      </c>
-      <c r="E6" s="7"/>
-      <c r="F6" s="9"/>
-      <c r="G6" s="9"/>
-      <c r="H6" s="10" t="str">
+        <v>lunes a viernes</v>
+      </c>
+      <c r="E6" s="7" t="s">
+        <v>94</v>
+      </c>
+      <c r="F6" s="9">
+        <v>46146</v>
+      </c>
+      <c r="G6" s="9">
+        <v>46149</v>
+      </c>
+      <c r="H6" s="10">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="I6" s="7" t="str">
-        <f t="shared" si="2"/>
-        <v/>
+        <v>4</v>
+      </c>
+      <c r="I6" s="7" t="s">
+        <v>52</v>
       </c>
       <c r="J6" s="7"/>
       <c r="K6" s="7" t="str">
         <f t="shared" si="0"/>
-        <v/>
+        <v>52|20260504|20260507</v>
       </c>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.3">
@@ -2111,7 +2158,7 @@
         <v/>
       </c>
       <c r="I7" s="7" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" ref="I5:I66" si="2">IF(A7="","","PENDIENTE")</f>
         <v/>
       </c>
       <c r="J7" s="7"/>
@@ -8160,7 +8207,7 @@
       <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="4">
         <x14:dataValidation type="list" xr:uid="{00000000-0002-0000-0200-000000000000}">
           <x14:formula1>
-            <xm:f>Empleados!$A$2:$A$29</xm:f>
+            <xm:f>Empleados!$A$3:$A$30</xm:f>
           </x14:formula1>
           <xm:sqref>A2:A201</xm:sqref>
         </x14:dataValidation>
@@ -8198,53 +8245,53 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="18" x14ac:dyDescent="0.35">
-      <c r="A1" s="12" t="s">
-        <v>78</v>
-      </c>
-      <c r="B1" s="13"/>
-      <c r="C1" s="13"/>
-      <c r="D1" s="13"/>
+      <c r="A1" s="13" t="s">
+        <v>77</v>
+      </c>
+      <c r="B1" s="14"/>
+      <c r="C1" s="14"/>
+      <c r="D1" s="14"/>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A3" s="6" t="s">
+        <v>78</v>
+      </c>
+      <c r="B3" s="6" t="s">
         <v>79</v>
       </c>
-      <c r="B3" s="6" t="s">
+      <c r="D3" s="6" t="s">
         <v>80</v>
       </c>
-      <c r="D3" s="6" t="s">
+      <c r="E3" s="6" t="s">
         <v>81</v>
-      </c>
-      <c r="E3" s="6" t="s">
-        <v>82</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B4" s="8">
         <f>COUNTA(Ausencias!A2:A201)</f>
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="D4" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="E4">
         <f>COUNTIF(Ausencias!E2:E201,"VACACIONES")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="B5" s="8">
         <f>SUM(Ausencias!H2:H201)</f>
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="D5" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="E5">
         <f>COUNTIF(Ausencias!E2:E201,"ENFERMEDAD")</f>
@@ -8253,14 +8300,14 @@
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="B6" s="8">
         <f>COUNTIF(Ausencias!I2:I201,"PENDIENTE")</f>
         <v>0</v>
       </c>
       <c r="D6" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="E6">
         <f>COUNTIF(Ausencias!E2:E201,"ART")</f>
@@ -8269,14 +8316,14 @@
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="B7" s="8">
         <f>COUNTIF(Ausencias!I2:I201,"APROBADO")</f>
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="D7" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="E7">
         <f>COUNTIF(Ausencias!E2:E201,"PERMISO")</f>
@@ -8285,14 +8332,14 @@
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="B8" s="8">
         <f>COUNTIF(Ausencias!E2:E201,"VACACIONES")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D8" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="E8">
         <f>COUNTIF(Ausencias!E2:E201,"FRANCO")</f>
@@ -8301,16 +8348,16 @@
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.3">
       <c r="D9" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E9">
         <f>COUNTIF(Ausencias!E2:E201,"FERIADO")</f>
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.3">
       <c r="D10" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="E10">
         <f>COUNTIF(Ausencias!E2:E201,"HOME OFFICE")</f>
@@ -8319,7 +8366,7 @@
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.3">
       <c r="D11" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="E11">
         <f>COUNTIF(Ausencias!E2:E201,"SUSPENSION")</f>
@@ -8328,7 +8375,7 @@
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.3">
       <c r="D12" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="E12">
         <f>COUNTIF(Ausencias!E2:E201,"AUSENCIA JUSTIFICADA")</f>
@@ -8337,7 +8384,7 @@
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.3">
       <c r="D13" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="E13">
         <f>COUNTIF(Ausencias!E2:E201,"OTRO")</f>

</xml_diff>

<commit_message>
actualizacion de interface UI y manual de usuario
</commit_message>
<xml_diff>
--- a/date.xlsx
+++ b/date.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Lucas\Desktop\hikvision-hours-processor\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6856CA0F-E158-41BE-85AB-1704C5BEBCD1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DAFC57DC-D512-4109-8BDF-DD152A68A46E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Empleados" sheetId="1" r:id="rId1"/>
@@ -2045,11 +2045,11 @@
         <v>46146</v>
       </c>
       <c r="G4" s="9">
-        <v>46149</v>
+        <v>46157</v>
       </c>
       <c r="H4" s="10">
         <f t="shared" si="1"/>
-        <v>4</v>
+        <v>12</v>
       </c>
       <c r="I4" s="7" t="s">
         <v>52</v>
@@ -2057,7 +2057,7 @@
       <c r="J4" s="7"/>
       <c r="K4" s="7" t="str">
         <f t="shared" si="0"/>
-        <v>82|20260504|20260507</v>
+        <v>82|20260504|20260515</v>
       </c>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.3">
@@ -2083,11 +2083,11 @@
         <v>46146</v>
       </c>
       <c r="G5" s="9">
-        <v>46149</v>
+        <v>46157</v>
       </c>
       <c r="H5" s="10">
         <f t="shared" si="1"/>
-        <v>4</v>
+        <v>12</v>
       </c>
       <c r="I5" s="7" t="s">
         <v>52</v>
@@ -2095,7 +2095,7 @@
       <c r="J5" s="7"/>
       <c r="K5" s="7" t="str">
         <f t="shared" si="0"/>
-        <v>52|20260504|20260507</v>
+        <v>52|20260504|20260515</v>
       </c>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.3">
@@ -8250,7 +8250,7 @@
       </c>
       <c r="B5" s="8">
         <f>SUM(Ausencias!H2:H200)</f>
-        <v>10</v>
+        <v>26</v>
       </c>
       <c r="D5" t="s">
         <v>51</v>

</xml_diff>

<commit_message>
cambio en reporte "liquidar", separacion por quincena
</commit_message>
<xml_diff>
--- a/date.xlsx
+++ b/date.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Lucas\Desktop\hikvision-hours-processor\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DAFC57DC-D512-4109-8BDF-DD152A68A46E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{ECDEF3F1-995F-4B71-8C8B-C56407BE00F4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Empleados" sheetId="1" r:id="rId1"/>
@@ -2045,11 +2045,11 @@
         <v>46146</v>
       </c>
       <c r="G4" s="9">
-        <v>46157</v>
+        <v>46173</v>
       </c>
       <c r="H4" s="10">
         <f t="shared" si="1"/>
-        <v>12</v>
+        <v>28</v>
       </c>
       <c r="I4" s="7" t="s">
         <v>52</v>
@@ -2057,7 +2057,7 @@
       <c r="J4" s="7"/>
       <c r="K4" s="7" t="str">
         <f t="shared" si="0"/>
-        <v>82|20260504|20260515</v>
+        <v>82|20260504|20260531</v>
       </c>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.3">
@@ -2083,11 +2083,11 @@
         <v>46146</v>
       </c>
       <c r="G5" s="9">
-        <v>46157</v>
+        <v>46173</v>
       </c>
       <c r="H5" s="10">
         <f t="shared" si="1"/>
-        <v>12</v>
+        <v>28</v>
       </c>
       <c r="I5" s="7" t="s">
         <v>52</v>
@@ -2095,7 +2095,7 @@
       <c r="J5" s="7"/>
       <c r="K5" s="7" t="str">
         <f t="shared" si="0"/>
-        <v>52|20260504|20260515</v>
+        <v>52|20260504|20260531</v>
       </c>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.3">
@@ -8250,7 +8250,7 @@
       </c>
       <c r="B5" s="8">
         <f>SUM(Ausencias!H2:H200)</f>
-        <v>26</v>
+        <v>58</v>
       </c>
       <c r="D5" t="s">
         <v>51</v>

</xml_diff>

<commit_message>
se agrego resumen de tardanzas y ausencias.
</commit_message>
<xml_diff>
--- a/date.xlsx
+++ b/date.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Lucas\Desktop\hikvision-hours-processor\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DB020003-D8C3-4627-8CE1-127746A8E342}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1854E517-6919-47C6-B750-057A9E570854}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Empleados" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="175" uniqueCount="96">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="177" uniqueCount="96">
   <si>
     <t>Id</t>
   </si>
@@ -606,7 +606,7 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>1</c:v>
+                  <c:v>2</c:v>
                 </c:pt>
                 <c:pt idx="6">
                   <c:v>0</c:v>
@@ -2074,34 +2074,41 @@
       </c>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A6" s="7"/>
+      <c r="A6" s="7">
+        <v>1</v>
+      </c>
       <c r="B6" s="7" t="str">
         <f>IF(A6="","",IFERROR(VLOOKUP(A6,Empleados!A:B,2,FALSE),""))</f>
-        <v/>
-      </c>
-      <c r="C6" s="7" t="str">
+        <v>Todos</v>
+      </c>
+      <c r="C6" s="7">
         <f>IF(A6="","",IFERROR(VLOOKUP(A6,Empleados!A:I,9,FALSE),""))</f>
-        <v/>
-      </c>
-      <c r="D6" s="7" t="str">
+        <v>0</v>
+      </c>
+      <c r="D6" s="7">
         <f>IF(A6="","",IFERROR(VLOOKUP(A6,Empleados!A:H,8,FALSE),""))</f>
-        <v/>
-      </c>
-      <c r="E6" s="7"/>
-      <c r="F6" s="9"/>
-      <c r="G6" s="9"/>
-      <c r="H6" s="10" t="str">
+        <v>0</v>
+      </c>
+      <c r="E6" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="F6" s="9">
+        <v>46167</v>
+      </c>
+      <c r="G6" s="9">
+        <v>46167</v>
+      </c>
+      <c r="H6" s="10">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="I6" s="7" t="str">
-        <f t="shared" ref="I6:I65" si="2">IF(A6="","","PENDIENTE")</f>
-        <v/>
+        <v>1</v>
+      </c>
+      <c r="I6" s="7" t="s">
+        <v>51</v>
       </c>
       <c r="J6" s="7"/>
       <c r="K6" s="7" t="str">
         <f t="shared" si="0"/>
-        <v/>
+        <v>1|20260525|20260525</v>
       </c>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.3">
@@ -2126,7 +2133,7 @@
         <v/>
       </c>
       <c r="I7" s="7" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" ref="I6:I65" si="2">IF(A7="","","PENDIENTE")</f>
         <v/>
       </c>
       <c r="J7" s="7"/>
@@ -8209,7 +8216,7 @@
       </c>
       <c r="B4" s="8">
         <f>COUNTA(Ausencias!A2:A200)</f>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D4" t="s">
         <v>47</v>
@@ -8225,7 +8232,7 @@
       </c>
       <c r="B5" s="8">
         <f>SUM(Ausencias!H2:H200)</f>
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D5" t="s">
         <v>50</v>
@@ -8257,7 +8264,7 @@
       </c>
       <c r="B7" s="8">
         <f>COUNTIF(Ausencias!I2:I200,"APROBADO")</f>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D7" t="s">
         <v>56</v>
@@ -8289,7 +8296,7 @@
       </c>
       <c r="E9">
         <f>COUNTIF(Ausencias!E2:E200,"FERIADO")</f>
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
Agrega hojas Tardanzas y Resumen; mejoras varias
</commit_message>
<xml_diff>
--- a/date.xlsx
+++ b/date.xlsx
@@ -1,25 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="600" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-105" yWindow="-105" windowWidth="23250" windowHeight="12450" tabRatio="600" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Empleados" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Ausencias" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Config" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Empleados" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ausencias" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Config" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="191029" fullCalcOnLoad="1"/>
+  <calcPr calcId="162913" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="dd/mm/yyyy"/>
-  </numFmts>
+  <numFmts count="0"/>
   <fonts count="4">
     <font>
       <name val="Calibri"/>
@@ -100,7 +98,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
@@ -123,7 +121,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -135,11 +133,23 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="7">
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
     <dxf>
       <fill>
         <patternFill patternType="solid">
@@ -167,15 +177,6 @@
           <bgColor rgb="FFD9EAF7"/>
         </patternFill>
       </fill>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -268,16 +269,16 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="TablaAusencias" displayName="TablaAusencias" ref="A1:K198" headerRowCount="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="TablaAusencias" displayName="TablaAusencias" ref="A1:K197" headerRowCount="1">
   <tableColumns count="11">
     <tableColumn id="1" name="Legajo"/>
-    <tableColumn id="2" name="Nombre (auto)" dataDxfId="6">
+    <tableColumn id="2" name="Nombre (auto)" dataDxfId="2">
       <calculatedColumnFormula>IF(A2="","",IFERROR(VLOOKUP(A2,Empleados!A:B,2,FALSE),""))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" name="Grupo (auto)" dataDxfId="5">
+    <tableColumn id="3" name="Grupo (auto)" dataDxfId="1">
       <calculatedColumnFormula>IF(A2="","",IFERROR(VLOOKUP(A2,Empleados!A:I,9,FALSE),""))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" name="Días laborales (auto)" dataDxfId="4">
+    <tableColumn id="4" name="Días laborales (auto)" dataDxfId="0">
       <calculatedColumnFormula>IF(A2="","",IFERROR(VLOOKUP(A2,Empleados!A:H,8,FALSE),""))</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="6" name="Tipo ausencia"/>
@@ -450,17 +451,17 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:I1048570"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" style="1" min="1" max="1"/>
     <col width="28" customWidth="1" style="1" min="2" max="2"/>
     <col width="18" customWidth="1" style="1" min="3" max="6"/>
     <col width="16" customWidth="1" style="1" min="7" max="7"/>
-    <col width="22.21875" bestFit="1" customWidth="1" style="1" min="8" max="8"/>
+    <col width="22.28515625" bestFit="1" customWidth="1" style="1" min="8" max="8"/>
     <col width="20" customWidth="1" style="1" min="9" max="9"/>
   </cols>
   <sheetData>
-    <row r="1" ht="28.8" customHeight="1">
+    <row r="1" ht="28.9" customHeight="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
           <t>Id</t>
@@ -1496,8 +1497,8 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K198"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
+  <dimension ref="A1:K197"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="28" customWidth="1" min="2" max="2"/>
@@ -1568,7 +1569,7 @@
     </row>
     <row r="2">
       <c r="A2" s="7" t="n">
-        <v>100</v>
+        <v>1</v>
       </c>
       <c r="B2" s="7">
         <f>IF(A2="","",IFERROR(VLOOKUP(A2,Empleados!A:B,2,FALSE),""))</f>
@@ -1584,14 +1585,14 @@
       </c>
       <c r="E2" s="7" t="inlineStr">
         <is>
-          <t>VACACIONES</t>
+          <t>FERIADO</t>
         </is>
       </c>
       <c r="F2" s="8" t="n">
-        <v>46140</v>
+        <v>46143</v>
       </c>
       <c r="G2" s="8" t="n">
-        <v>46140</v>
+        <v>46143</v>
       </c>
       <c r="H2" s="9">
         <f>IF(OR(F2="",G2=""),"",G2-F2+1)</f>
@@ -1608,9 +1609,9 @@
         <v/>
       </c>
     </row>
-    <row r="3">
+    <row r="3" ht="30.75" customHeight="1">
       <c r="A3" s="7" t="n">
-        <v>1</v>
+        <v>82</v>
       </c>
       <c r="B3" s="7">
         <f>IF(A3="","",IFERROR(VLOOKUP(A3,Empleados!A:B,2,FALSE),""))</f>
@@ -1626,14 +1627,14 @@
       </c>
       <c r="E3" s="7" t="inlineStr">
         <is>
-          <t>FERIADO</t>
+          <t>ACCIDENTE DE TRABAJO</t>
         </is>
       </c>
       <c r="F3" s="8" t="n">
-        <v>46143</v>
+        <v>46146</v>
       </c>
       <c r="G3" s="8" t="n">
-        <v>46143</v>
+        <v>46173</v>
       </c>
       <c r="H3" s="9">
         <f>IF(OR(F3="",G3=""),"",G3-F3+1)</f>
@@ -1650,9 +1651,9 @@
         <v/>
       </c>
     </row>
-    <row r="4">
+    <row r="4" ht="13.5" customHeight="1">
       <c r="A4" s="7" t="n">
-        <v>82</v>
+        <v>52</v>
       </c>
       <c r="B4" s="7">
         <f>IF(A4="","",IFERROR(VLOOKUP(A4,Empleados!A:B,2,FALSE),""))</f>
@@ -1694,7 +1695,7 @@
     </row>
     <row r="5">
       <c r="A5" s="7" t="n">
-        <v>52</v>
+        <v>1</v>
       </c>
       <c r="B5" s="7">
         <f>IF(A5="","",IFERROR(VLOOKUP(A5,Empleados!A:B,2,FALSE),""))</f>
@@ -1710,14 +1711,14 @@
       </c>
       <c r="E5" s="7" t="inlineStr">
         <is>
-          <t>ACCIDENTE DE TRABAJO</t>
+          <t>FERIADO</t>
         </is>
       </c>
       <c r="F5" s="8" t="n">
-        <v>46146</v>
+        <v>46167</v>
       </c>
       <c r="G5" s="8" t="n">
-        <v>46173</v>
+        <v>46167</v>
       </c>
       <c r="H5" s="9">
         <f>IF(OR(F5="",G5=""),"",G5-F5+1)</f>
@@ -1736,7 +1737,7 @@
     </row>
     <row r="6">
       <c r="A6" s="7" t="n">
-        <v>1</v>
+        <v>93</v>
       </c>
       <c r="B6" s="7">
         <f>IF(A6="","",IFERROR(VLOOKUP(A6,Empleados!A:B,2,FALSE),""))</f>
@@ -1752,14 +1753,14 @@
       </c>
       <c r="E6" s="7" t="inlineStr">
         <is>
-          <t>FERIADO</t>
+          <t>PRESENTE</t>
         </is>
       </c>
       <c r="F6" s="8" t="n">
-        <v>46167</v>
+        <v>46149</v>
       </c>
       <c r="G6" s="8" t="n">
-        <v>46167</v>
+        <v>46156</v>
       </c>
       <c r="H6" s="9">
         <f>IF(OR(F6="",G6=""),"",G6-F6+1)</f>
@@ -1778,7 +1779,7 @@
     </row>
     <row r="7">
       <c r="A7" s="7" t="n">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="B7" s="7">
         <f>IF(A7="","",IFERROR(VLOOKUP(A7,Empleados!A:B,2,FALSE),""))</f>
@@ -1798,10 +1799,10 @@
         </is>
       </c>
       <c r="F7" s="8" t="n">
-        <v>46149</v>
+        <v>46156</v>
       </c>
       <c r="G7" s="8" t="n">
-        <v>46156</v>
+        <v>46157</v>
       </c>
       <c r="H7" s="9">
         <f>IF(OR(F7="",G7=""),"",G7-F7+1)</f>
@@ -1820,7 +1821,7 @@
     </row>
     <row r="8">
       <c r="A8" s="7" t="n">
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="B8" s="7">
         <f>IF(A8="","",IFERROR(VLOOKUP(A8,Empleados!A:B,2,FALSE),""))</f>
@@ -1840,10 +1841,10 @@
         </is>
       </c>
       <c r="F8" s="8" t="n">
-        <v>46156</v>
+        <v>46154</v>
       </c>
       <c r="G8" s="8" t="n">
-        <v>46157</v>
+        <v>46155</v>
       </c>
       <c r="H8" s="9">
         <f>IF(OR(F8="",G8=""),"",G8-F8+1)</f>
@@ -1862,7 +1863,7 @@
     </row>
     <row r="9">
       <c r="A9" s="7" t="n">
-        <v>100</v>
+        <v>51</v>
       </c>
       <c r="B9" s="7">
         <f>IF(A9="","",IFERROR(VLOOKUP(A9,Empleados!A:B,2,FALSE),""))</f>
@@ -1878,14 +1879,14 @@
       </c>
       <c r="E9" s="7" t="inlineStr">
         <is>
-          <t>PRESENTE</t>
+          <t>AUSENCIA</t>
         </is>
       </c>
       <c r="F9" s="8" t="n">
-        <v>46154</v>
+        <v>46161</v>
       </c>
       <c r="G9" s="8" t="n">
-        <v>46155</v>
+        <v>46161</v>
       </c>
       <c r="H9" s="9">
         <f>IF(OR(F9="",G9=""),"",G9-F9+1)</f>
@@ -1903,7 +1904,9 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="7" t="n"/>
+      <c r="A10" s="7" t="n">
+        <v>51</v>
+      </c>
       <c r="B10" s="7">
         <f>IF(A10="","",IFERROR(VLOOKUP(A10,Empleados!A:B,2,FALSE),""))</f>
         <v/>
@@ -1916,16 +1919,25 @@
         <f>IF(A10="","",IFERROR(VLOOKUP(A10,Empleados!A:H,8,FALSE),""))</f>
         <v/>
       </c>
-      <c r="E10" s="7" t="n"/>
-      <c r="F10" s="8" t="n"/>
-      <c r="G10" s="8" t="n"/>
+      <c r="E10" s="7" t="inlineStr">
+        <is>
+          <t>PRESENTE</t>
+        </is>
+      </c>
+      <c r="F10" s="8" t="n">
+        <v>46154</v>
+      </c>
+      <c r="G10" s="8" t="n">
+        <v>46156</v>
+      </c>
       <c r="H10" s="9">
         <f>IF(OR(F10="",G10=""),"",G10-F10+1)</f>
         <v/>
       </c>
-      <c r="I10" s="7">
-        <f>IF(A10="","","PENDIENTE")</f>
-        <v/>
+      <c r="I10" s="7" t="inlineStr">
+        <is>
+          <t>APROBADO</t>
+        </is>
       </c>
       <c r="J10" s="7" t="n"/>
       <c r="K10" s="7">
@@ -1934,7 +1946,9 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="7" t="n"/>
+      <c r="A11" s="7" t="n">
+        <v>20</v>
+      </c>
       <c r="B11" s="7">
         <f>IF(A11="","",IFERROR(VLOOKUP(A11,Empleados!A:B,2,FALSE),""))</f>
         <v/>
@@ -1947,16 +1961,25 @@
         <f>IF(A11="","",IFERROR(VLOOKUP(A11,Empleados!A:H,8,FALSE),""))</f>
         <v/>
       </c>
-      <c r="E11" s="7" t="n"/>
-      <c r="F11" s="8" t="n"/>
-      <c r="G11" s="8" t="n"/>
+      <c r="E11" s="7" t="inlineStr">
+        <is>
+          <t>VACACIONES</t>
+        </is>
+      </c>
+      <c r="F11" s="8" t="n">
+        <v>46164</v>
+      </c>
+      <c r="G11" s="8" t="n">
+        <v>46164</v>
+      </c>
       <c r="H11" s="9">
         <f>IF(OR(F11="",G11=""),"",G11-F11+1)</f>
         <v/>
       </c>
-      <c r="I11" s="7">
-        <f>IF(A11="","","PENDIENTE")</f>
-        <v/>
+      <c r="I11" s="7" t="inlineStr">
+        <is>
+          <t>APROBADO</t>
+        </is>
       </c>
       <c r="J11" s="7" t="n"/>
       <c r="K11" s="7">
@@ -1965,7 +1988,9 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="7" t="n"/>
+      <c r="A12" s="7" t="n">
+        <v>20</v>
+      </c>
       <c r="B12" s="7">
         <f>IF(A12="","",IFERROR(VLOOKUP(A12,Empleados!A:B,2,FALSE),""))</f>
         <v/>
@@ -1978,16 +2003,25 @@
         <f>IF(A12="","",IFERROR(VLOOKUP(A12,Empleados!A:H,8,FALSE),""))</f>
         <v/>
       </c>
-      <c r="E12" s="7" t="n"/>
-      <c r="F12" s="8" t="n"/>
-      <c r="G12" s="8" t="n"/>
+      <c r="E12" s="7" t="inlineStr">
+        <is>
+          <t>PRESENTE</t>
+        </is>
+      </c>
+      <c r="F12" s="8" t="n">
+        <v>46170</v>
+      </c>
+      <c r="G12" s="8" t="n">
+        <v>46170</v>
+      </c>
       <c r="H12" s="9">
         <f>IF(OR(F12="",G12=""),"",G12-F12+1)</f>
         <v/>
       </c>
-      <c r="I12" s="7">
-        <f>IF(A12="","","PENDIENTE")</f>
-        <v/>
+      <c r="I12" s="7" t="inlineStr">
+        <is>
+          <t>APROBADO</t>
+        </is>
       </c>
       <c r="J12" s="7" t="n"/>
       <c r="K12" s="7">
@@ -1996,7 +2030,9 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="7" t="n"/>
+      <c r="A13" s="7" t="n">
+        <v>97</v>
+      </c>
       <c r="B13" s="7">
         <f>IF(A13="","",IFERROR(VLOOKUP(A13,Empleados!A:B,2,FALSE),""))</f>
         <v/>
@@ -2009,16 +2045,25 @@
         <f>IF(A13="","",IFERROR(VLOOKUP(A13,Empleados!A:H,8,FALSE),""))</f>
         <v/>
       </c>
-      <c r="E13" s="7" t="n"/>
-      <c r="F13" s="8" t="n"/>
-      <c r="G13" s="8" t="n"/>
+      <c r="E13" s="7" t="inlineStr">
+        <is>
+          <t>PRESENTE</t>
+        </is>
+      </c>
+      <c r="F13" s="8" t="n">
+        <v>46168</v>
+      </c>
+      <c r="G13" s="8" t="n">
+        <v>46169</v>
+      </c>
       <c r="H13" s="9">
         <f>IF(OR(F13="",G13=""),"",G13-F13+1)</f>
         <v/>
       </c>
-      <c r="I13" s="7">
-        <f>IF(A13="","","PENDIENTE")</f>
-        <v/>
+      <c r="I13" s="7" t="inlineStr">
+        <is>
+          <t>APROBADO</t>
+        </is>
       </c>
       <c r="J13" s="7" t="n"/>
       <c r="K13" s="7">
@@ -2027,7 +2072,9 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="7" t="n"/>
+      <c r="A14" s="7" t="n">
+        <v>96</v>
+      </c>
       <c r="B14" s="7">
         <f>IF(A14="","",IFERROR(VLOOKUP(A14,Empleados!A:B,2,FALSE),""))</f>
         <v/>
@@ -2040,16 +2087,25 @@
         <f>IF(A14="","",IFERROR(VLOOKUP(A14,Empleados!A:H,8,FALSE),""))</f>
         <v/>
       </c>
-      <c r="E14" s="7" t="n"/>
-      <c r="F14" s="8" t="n"/>
-      <c r="G14" s="8" t="n"/>
+      <c r="E14" s="7" t="inlineStr">
+        <is>
+          <t>PRESENTE</t>
+        </is>
+      </c>
+      <c r="F14" s="8" t="n">
+        <v>46168</v>
+      </c>
+      <c r="G14" s="8" t="n">
+        <v>46169</v>
+      </c>
       <c r="H14" s="9">
         <f>IF(OR(F14="",G14=""),"",G14-F14+1)</f>
         <v/>
       </c>
-      <c r="I14" s="7">
-        <f>IF(A14="","","PENDIENTE")</f>
-        <v/>
+      <c r="I14" s="7" t="inlineStr">
+        <is>
+          <t>APROBADO</t>
+        </is>
       </c>
       <c r="J14" s="7" t="n"/>
       <c r="K14" s="7">
@@ -2058,7 +2114,9 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="7" t="n"/>
+      <c r="A15" s="7" t="n">
+        <v>100</v>
+      </c>
       <c r="B15" s="7">
         <f>IF(A15="","",IFERROR(VLOOKUP(A15,Empleados!A:B,2,FALSE),""))</f>
         <v/>
@@ -2071,16 +2129,25 @@
         <f>IF(A15="","",IFERROR(VLOOKUP(A15,Empleados!A:H,8,FALSE),""))</f>
         <v/>
       </c>
-      <c r="E15" s="7" t="n"/>
-      <c r="F15" s="8" t="n"/>
-      <c r="G15" s="8" t="n"/>
+      <c r="E15" s="7" t="inlineStr">
+        <is>
+          <t>PRESENTE</t>
+        </is>
+      </c>
+      <c r="F15" s="8" t="n">
+        <v>46157</v>
+      </c>
+      <c r="G15" s="8" t="n">
+        <v>46157</v>
+      </c>
       <c r="H15" s="9">
         <f>IF(OR(F15="",G15=""),"",G15-F15+1)</f>
         <v/>
       </c>
-      <c r="I15" s="7">
-        <f>IF(A15="","","PENDIENTE")</f>
-        <v/>
+      <c r="I15" s="7" t="inlineStr">
+        <is>
+          <t>APROBADO</t>
+        </is>
       </c>
       <c r="J15" s="7" t="n"/>
       <c r="K15" s="7">
@@ -2089,7 +2156,9 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="7" t="n"/>
+      <c r="A16" s="7" t="n">
+        <v>113</v>
+      </c>
       <c r="B16" s="7">
         <f>IF(A16="","",IFERROR(VLOOKUP(A16,Empleados!A:B,2,FALSE),""))</f>
         <v/>
@@ -2102,16 +2171,25 @@
         <f>IF(A16="","",IFERROR(VLOOKUP(A16,Empleados!A:H,8,FALSE),""))</f>
         <v/>
       </c>
-      <c r="E16" s="7" t="n"/>
-      <c r="F16" s="8" t="n"/>
-      <c r="G16" s="8" t="n"/>
+      <c r="E16" s="7" t="inlineStr">
+        <is>
+          <t>PRESENTE</t>
+        </is>
+      </c>
+      <c r="F16" s="8" t="n">
+        <v>46154</v>
+      </c>
+      <c r="G16" s="8" t="n">
+        <v>46154</v>
+      </c>
       <c r="H16" s="9">
         <f>IF(OR(F16="",G16=""),"",G16-F16+1)</f>
         <v/>
       </c>
-      <c r="I16" s="7">
-        <f>IF(A16="","","PENDIENTE")</f>
-        <v/>
+      <c r="I16" s="7" t="inlineStr">
+        <is>
+          <t>APROBADO</t>
+        </is>
       </c>
       <c r="J16" s="7" t="n"/>
       <c r="K16" s="7">
@@ -2120,7 +2198,9 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="7" t="n"/>
+      <c r="A17" s="7" t="n">
+        <v>113</v>
+      </c>
       <c r="B17" s="7">
         <f>IF(A17="","",IFERROR(VLOOKUP(A17,Empleados!A:B,2,FALSE),""))</f>
         <v/>
@@ -2133,16 +2213,25 @@
         <f>IF(A17="","",IFERROR(VLOOKUP(A17,Empleados!A:H,8,FALSE),""))</f>
         <v/>
       </c>
-      <c r="E17" s="7" t="n"/>
-      <c r="F17" s="8" t="n"/>
-      <c r="G17" s="8" t="n"/>
+      <c r="E17" s="7" t="inlineStr">
+        <is>
+          <t>PRESENTE</t>
+        </is>
+      </c>
+      <c r="F17" s="8" t="n">
+        <v>46157</v>
+      </c>
+      <c r="G17" s="8" t="n">
+        <v>46157</v>
+      </c>
       <c r="H17" s="9">
         <f>IF(OR(F17="",G17=""),"",G17-F17+1)</f>
         <v/>
       </c>
-      <c r="I17" s="7">
-        <f>IF(A17="","","PENDIENTE")</f>
-        <v/>
+      <c r="I17" s="7" t="inlineStr">
+        <is>
+          <t>APROBADO</t>
+        </is>
       </c>
       <c r="J17" s="7" t="n"/>
       <c r="K17" s="7">
@@ -2151,7 +2240,9 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="7" t="n"/>
+      <c r="A18" s="7" t="n">
+        <v>113</v>
+      </c>
       <c r="B18" s="7">
         <f>IF(A18="","",IFERROR(VLOOKUP(A18,Empleados!A:B,2,FALSE),""))</f>
         <v/>
@@ -2164,16 +2255,25 @@
         <f>IF(A18="","",IFERROR(VLOOKUP(A18,Empleados!A:H,8,FALSE),""))</f>
         <v/>
       </c>
-      <c r="E18" s="7" t="n"/>
-      <c r="F18" s="8" t="n"/>
-      <c r="G18" s="8" t="n"/>
+      <c r="E18" s="7" t="inlineStr">
+        <is>
+          <t>AUSENCIA</t>
+        </is>
+      </c>
+      <c r="F18" s="8" t="n">
+        <v>46164</v>
+      </c>
+      <c r="G18" s="8" t="n">
+        <v>46164</v>
+      </c>
       <c r="H18" s="9">
         <f>IF(OR(F18="",G18=""),"",G18-F18+1)</f>
         <v/>
       </c>
-      <c r="I18" s="7">
-        <f>IF(A18="","","PENDIENTE")</f>
-        <v/>
+      <c r="I18" s="7" t="inlineStr">
+        <is>
+          <t>APROBADO</t>
+        </is>
       </c>
       <c r="J18" s="7" t="n"/>
       <c r="K18" s="7">
@@ -2182,7 +2282,9 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="7" t="n"/>
+      <c r="A19" s="7" t="n">
+        <v>109</v>
+      </c>
       <c r="B19" s="7">
         <f>IF(A19="","",IFERROR(VLOOKUP(A19,Empleados!A:B,2,FALSE),""))</f>
         <v/>
@@ -2195,16 +2297,25 @@
         <f>IF(A19="","",IFERROR(VLOOKUP(A19,Empleados!A:H,8,FALSE),""))</f>
         <v/>
       </c>
-      <c r="E19" s="7" t="n"/>
-      <c r="F19" s="8" t="n"/>
-      <c r="G19" s="8" t="n"/>
+      <c r="E19" s="7" t="inlineStr">
+        <is>
+          <t>PRESENTE</t>
+        </is>
+      </c>
+      <c r="F19" s="8" t="n">
+        <v>46169</v>
+      </c>
+      <c r="G19" s="8" t="n">
+        <v>46170</v>
+      </c>
       <c r="H19" s="9">
         <f>IF(OR(F19="",G19=""),"",G19-F19+1)</f>
         <v/>
       </c>
-      <c r="I19" s="7">
-        <f>IF(A19="","","PENDIENTE")</f>
-        <v/>
+      <c r="I19" s="7" t="inlineStr">
+        <is>
+          <t>APROBADO</t>
+        </is>
       </c>
       <c r="J19" s="7" t="n"/>
       <c r="K19" s="7">
@@ -2213,7 +2324,9 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="7" t="n"/>
+      <c r="A20" s="7" t="n">
+        <v>83</v>
+      </c>
       <c r="B20" s="7">
         <f>IF(A20="","",IFERROR(VLOOKUP(A20,Empleados!A:B,2,FALSE),""))</f>
         <v/>
@@ -2226,16 +2339,25 @@
         <f>IF(A20="","",IFERROR(VLOOKUP(A20,Empleados!A:H,8,FALSE),""))</f>
         <v/>
       </c>
-      <c r="E20" s="7" t="n"/>
-      <c r="F20" s="8" t="n"/>
-      <c r="G20" s="8" t="n"/>
+      <c r="E20" s="7" t="inlineStr">
+        <is>
+          <t>PRESENTE</t>
+        </is>
+      </c>
+      <c r="F20" s="8" t="n">
+        <v>46156</v>
+      </c>
+      <c r="G20" s="8" t="n">
+        <v>46156</v>
+      </c>
       <c r="H20" s="9">
         <f>IF(OR(F20="",G20=""),"",G20-F20+1)</f>
         <v/>
       </c>
-      <c r="I20" s="7">
-        <f>IF(A20="","","PENDIENTE")</f>
-        <v/>
+      <c r="I20" s="7" t="inlineStr">
+        <is>
+          <t>APROBADO</t>
+        </is>
       </c>
       <c r="J20" s="7" t="n"/>
       <c r="K20" s="7">
@@ -2244,7 +2366,9 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="7" t="n"/>
+      <c r="A21" s="7" t="n">
+        <v>109</v>
+      </c>
       <c r="B21" s="7">
         <f>IF(A21="","",IFERROR(VLOOKUP(A21,Empleados!A:B,2,FALSE),""))</f>
         <v/>
@@ -2257,16 +2381,25 @@
         <f>IF(A21="","",IFERROR(VLOOKUP(A21,Empleados!A:H,8,FALSE),""))</f>
         <v/>
       </c>
-      <c r="E21" s="7" t="n"/>
-      <c r="F21" s="8" t="n"/>
-      <c r="G21" s="8" t="n"/>
+      <c r="E21" s="7" t="inlineStr">
+        <is>
+          <t>PRESENTE</t>
+        </is>
+      </c>
+      <c r="F21" s="8" t="n">
+        <v>46146</v>
+      </c>
+      <c r="G21" s="8" t="n">
+        <v>46146</v>
+      </c>
       <c r="H21" s="9">
         <f>IF(OR(F21="",G21=""),"",G21-F21+1)</f>
         <v/>
       </c>
-      <c r="I21" s="7">
-        <f>IF(A21="","","PENDIENTE")</f>
-        <v/>
+      <c r="I21" s="7" t="inlineStr">
+        <is>
+          <t>APROBADO</t>
+        </is>
       </c>
       <c r="J21" s="7" t="n"/>
       <c r="K21" s="7">
@@ -2275,7 +2408,9 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="7" t="n"/>
+      <c r="A22" s="7" t="n">
+        <v>120</v>
+      </c>
       <c r="B22" s="7">
         <f>IF(A22="","",IFERROR(VLOOKUP(A22,Empleados!A:B,2,FALSE),""))</f>
         <v/>
@@ -2288,16 +2423,25 @@
         <f>IF(A22="","",IFERROR(VLOOKUP(A22,Empleados!A:H,8,FALSE),""))</f>
         <v/>
       </c>
-      <c r="E22" s="7" t="n"/>
-      <c r="F22" s="8" t="n"/>
-      <c r="G22" s="8" t="n"/>
+      <c r="E22" s="7" t="inlineStr">
+        <is>
+          <t>PRESENTE</t>
+        </is>
+      </c>
+      <c r="F22" s="8" t="n">
+        <v>46156</v>
+      </c>
+      <c r="G22" s="8" t="n">
+        <v>46156</v>
+      </c>
       <c r="H22" s="9">
         <f>IF(OR(F22="",G22=""),"",G22-F22+1)</f>
         <v/>
       </c>
-      <c r="I22" s="7">
-        <f>IF(A22="","","PENDIENTE")</f>
-        <v/>
+      <c r="I22" s="7" t="inlineStr">
+        <is>
+          <t>APROBADO</t>
+        </is>
       </c>
       <c r="J22" s="7" t="n"/>
       <c r="K22" s="7">
@@ -2306,7 +2450,9 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="7" t="n"/>
+      <c r="A23" s="7" t="n">
+        <v>121</v>
+      </c>
       <c r="B23" s="7">
         <f>IF(A23="","",IFERROR(VLOOKUP(A23,Empleados!A:B,2,FALSE),""))</f>
         <v/>
@@ -2319,16 +2465,25 @@
         <f>IF(A23="","",IFERROR(VLOOKUP(A23,Empleados!A:H,8,FALSE),""))</f>
         <v/>
       </c>
-      <c r="E23" s="7" t="n"/>
-      <c r="F23" s="8" t="n"/>
-      <c r="G23" s="8" t="n"/>
+      <c r="E23" s="14" t="inlineStr">
+        <is>
+          <t>PRESENTE</t>
+        </is>
+      </c>
+      <c r="F23" s="8" t="n">
+        <v>46156</v>
+      </c>
+      <c r="G23" s="8" t="n">
+        <v>46156</v>
+      </c>
       <c r="H23" s="9">
         <f>IF(OR(F23="",G23=""),"",G23-F23+1)</f>
         <v/>
       </c>
-      <c r="I23" s="7">
-        <f>IF(A23="","","PENDIENTE")</f>
-        <v/>
+      <c r="I23" s="7" t="inlineStr">
+        <is>
+          <t>APROBADO</t>
+        </is>
       </c>
       <c r="J23" s="7" t="n"/>
       <c r="K23" s="7">
@@ -7730,71 +7885,28 @@
         <v/>
       </c>
     </row>
-    <row r="198">
-      <c r="A198" s="7" t="n"/>
-      <c r="B198" s="7">
-        <f>IF(A198="","",IFERROR(VLOOKUP(A198,Empleados!A:B,2,FALSE),""))</f>
-        <v/>
-      </c>
-      <c r="C198" s="7">
-        <f>IF(A198="","",IFERROR(VLOOKUP(A198,Empleados!A:I,9,FALSE),""))</f>
-        <v/>
-      </c>
-      <c r="D198" s="7">
-        <f>IF(A198="","",IFERROR(VLOOKUP(A198,Empleados!A:H,8,FALSE),""))</f>
-        <v/>
-      </c>
-      <c r="E198" s="7" t="n"/>
-      <c r="F198" s="8" t="n"/>
-      <c r="G198" s="8" t="n"/>
-      <c r="H198" s="9">
-        <f>IF(OR(F198="",G198=""),"",G198-F198+1)</f>
-        <v/>
-      </c>
-      <c r="I198" s="7">
-        <f>IF(A198="","","PENDIENTE")</f>
-        <v/>
-      </c>
-      <c r="J198" s="7" t="n"/>
-      <c r="K198" s="7">
-        <f>IF(A198="","",A198&amp;"|"&amp;TEXT(F198,"yyyymmdd")&amp;"|"&amp;TEXT(G198,"yyyymmdd"))</f>
-        <v/>
-      </c>
-    </row>
   </sheetData>
-  <conditionalFormatting sqref="E2:E198">
-    <cfRule type="expression" priority="1" dxfId="3">
+  <conditionalFormatting sqref="E2:E197">
+    <cfRule type="expression" priority="1" dxfId="6">
       <formula>$E2="VACACIONES"</formula>
     </cfRule>
-    <cfRule type="expression" priority="2" dxfId="2">
+    <cfRule type="expression" priority="2" dxfId="5">
       <formula>$E2="ENFERMEDAD"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I2:I198">
-    <cfRule type="expression" priority="3" dxfId="1">
+  <conditionalFormatting sqref="I2:I197">
+    <cfRule type="expression" priority="3" dxfId="4">
       <formula>$I2="PENDIENTE"</formula>
     </cfRule>
-    <cfRule type="expression" priority="4" dxfId="0">
+    <cfRule type="expression" priority="4" dxfId="3">
       <formula>$I2="APROBADO"</formula>
     </cfRule>
   </conditionalFormatting>
-  <dataValidations count="8">
+  <dataValidations count="4">
     <dataValidation sqref="E2:E4999" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"DOMINGO,AUSENCIA,VACACIONES,ESTUDIAR,CAPACITACIONES,SUSPENCION,NO TRABAJADO,LICENCIA,FERIADO,ACCIDENTE DE TRABAJO,VIAJES,PRESENTE"</formula1>
     </dataValidation>
     <dataValidation sqref="I2:I4999" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"PENDIENTE,APROBADO,RECHAZADO"</formula1>
-    </dataValidation>
-    <dataValidation sqref="E2:E5000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"DOMINGO,AUSENCIA,VACACIONES,ESTUDIAR,CAPACITACIONES,SUSPENCION,NO TRABAJADO,LICENCIA,FERIADO,ACCIDENTE DE TRABAJO,VIAJES,PRESENTE"</formula1>
-    </dataValidation>
-    <dataValidation sqref="I2:I5000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"PENDIENTE,APROBADO,RECHAZADO"</formula1>
-    </dataValidation>
-    <dataValidation sqref="E2:E5000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"DOMINGO,AUSENCIA,VACACIONES,ESTUDIAR,CAPACITACIONES,SUSPENCION,NO TRABAJADO,LICENCIA,FERIADO,ACCIDENTE DE TRABAJO,VIAJES,PRESENTE"</formula1>
-    </dataValidation>
-    <dataValidation sqref="I2:I5000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"PENDIENTE,APROBADO,RECHAZADO"</formula1>
     </dataValidation>
     <dataValidation sqref="E2:E5000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
@@ -7818,7 +7930,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:E14"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
     <col width="20" customWidth="1" min="3" max="3"/>
@@ -7906,7 +8018,7 @@
         </is>
       </c>
     </row>
-    <row r="6">
+    <row r="6" ht="30" customHeight="1">
       <c r="A6" t="inlineStr">
         <is>
           <t>CAPACITACIONES</t>

</xml_diff>

<commit_message>
se eliminaron varias cosas
</commit_message>
<xml_diff>
--- a/date.xlsx
+++ b/date.xlsx
@@ -8056,7 +8056,13 @@
       <formula>$I2="APROBADO"</formula>
     </cfRule>
   </conditionalFormatting>
-  <dataValidations count="12">
+  <dataValidations count="14">
+    <dataValidation sqref="E2:E5000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"DOMINGO,AUSENCIA,VACACIONES,ESTUDIAR,CAPACITACIONES,SUSPENCION,NO TRABAJADO,LICENCIA,FERIADO,ACCIDENTE DE TRABAJO,VIAJES,PRESENTE"</formula1>
+    </dataValidation>
+    <dataValidation sqref="I2:I5000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"PENDIENTE,APROBADO,RECHAZADO"</formula1>
+    </dataValidation>
     <dataValidation sqref="E2:E5000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"DOMINGO,AUSENCIA,VACACIONES,ESTUDIAR,CAPACITACIONES,SUSPENCION,NO TRABAJADO,LICENCIA,FERIADO,ACCIDENTE DE TRABAJO,VIAJES,PRESENTE"</formula1>
     </dataValidation>

</xml_diff>